<commit_message>
Add 'More picks' tab: additional senior-care/healthcare guest-post targets
Adds a supplementary tab with 9 further on-audience candidates
(mobility/accessibility, veterans, nursing, healthcare-tech) surfaced
by broadened care-adjacent filtering, excluding the 133 already listed.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EyZhZSnP6QyNR5y5EJdqhU
</commit_message>
<xml_diff>
--- a/nursenextdoor-selected-links.xlsx
+++ b/nursenextdoor-selected-links.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="NurseNextDoor picks" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="More picks" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4451,4 +4452,344 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Focus</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>AS</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>TF</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Traffic</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>RD</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Price($)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>wheelchairtravel.org</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Accessibility / mobility</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>42</v>
+      </c>
+      <c r="D2" t="n">
+        <v>25</v>
+      </c>
+      <c r="E2" t="n">
+        <v>46903</v>
+      </c>
+      <c r="F2" t="n">
+        <v>3176</v>
+      </c>
+      <c r="G2" t="n">
+        <v>903</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>care-adjacent</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>usveteransmagazine.com</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Veterans (caregiving audience)</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>39</v>
+      </c>
+      <c r="D3" t="n">
+        <v>30</v>
+      </c>
+      <c r="E3" t="n">
+        <v>11753</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2784</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>nursekey.com</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Nursing reference</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>34</v>
+      </c>
+      <c r="D4" t="n">
+        <v>21</v>
+      </c>
+      <c r="E4" t="n">
+        <v>32527</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1960</v>
+      </c>
+      <c r="G4" t="n">
+        <v>220</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>good value</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>mobilita.org</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mobility</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>32</v>
+      </c>
+      <c r="D5" t="n">
+        <v>23</v>
+      </c>
+      <c r="E5" t="n">
+        <v>13110</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1086</v>
+      </c>
+      <c r="G5" t="n">
+        <v>210</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>good value</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>rightpatient.com</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Healthcare tech</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>31</v>
+      </c>
+      <c r="D6" t="n">
+        <v>26</v>
+      </c>
+      <c r="E6" t="n">
+        <v>5524</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1192</v>
+      </c>
+      <c r="G6" t="n">
+        <v>160</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>good value</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>medigy.com</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>31</v>
+      </c>
+      <c r="D7" t="n">
+        <v>25</v>
+      </c>
+      <c r="E7" t="n">
+        <v>3477</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1206</v>
+      </c>
+      <c r="G7" t="n">
+        <v>180</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>good value</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>briancolemd.com</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Medical advice</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>30</v>
+      </c>
+      <c r="D8" t="n">
+        <v>34</v>
+      </c>
+      <c r="E8" t="n">
+        <v>7240</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2362</v>
+      </c>
+      <c r="G8" t="n">
+        <v>120</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>good value</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>hospibuz.com</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Hospitals / healthcare</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>30</v>
+      </c>
+      <c r="D9" t="n">
+        <v>26</v>
+      </c>
+      <c r="E9" t="n">
+        <v>6026</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2497</v>
+      </c>
+      <c r="G9" t="n">
+        <v>210</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>good value</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>canhealth.com</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Canadian healthcare (NND is Canada-founded)</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>32</v>
+      </c>
+      <c r="D10" t="n">
+        <v>24</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2781</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1791</v>
+      </c>
+      <c r="G10" t="n">
+        <v>5665</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>pricey</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>